<commit_message>
Split rail/road into Inbound and Outbound, rename RMHS to Inbound, photos instead of drawn art
Each transport leg's rail/road slider now sits at the top of its own
department in plant customisation. RMHS is renamed Inbound in the Grid 5
workbook (applied by the calibration script), the site data, the code and
the tests. The drawn SVG art (department bands, panel art, hero art, database
preview) is removed and replaced with Unsplash photos: a banner per
department and a photo card for the database.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EeeEkUyyvv7aX46Z2Y1cVg
</commit_message>
<xml_diff>
--- a/data/source/Stainless_Steel_Carbon_Accounting_Grid_5.xlsx
+++ b/data/source/Stainless_Steel_Carbon_Accounting_Grid_5.xlsx
@@ -576,10 +576,11 @@
     <row r="2" ht="65" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Reference database of emission/energy formulas per process. Cells in Columns D-N are PLAIN TEXT formula ENTRIES (not live Excel formulas): x=virgin ratio, y=scrap ratio(=1-x); a-g = grid electricity source shares (Coal/Oil/Gas/Hydro/Wind/Solar/Nuclear, sum to 1); p=train share, q=road share(=1-p), used ONLY in the two Transport-related rows (RMHS&gt;Unloading/Inbound and Outbound&gt;Transport) — all other rows show N/A for p/q. See 'Grid Energy Mix Factors' sheet for a-g source factors. Only Scope 2 (Col P) varies with the energy mix; Scope 1, Scope 3(upstream), trace-gas columns and SEC do not. Column Q = Scope 3 UPSTREAM (GHG Protocol Cat. 1-8); downstream Cat. 9 is in Outbound &gt; Transport; Cat. 10-15 are in the 'Downstream Scope 3 (Product)' sheet. GWP basis: IPCC AR5 (100-yr). GRID 5: coefficients recalibrated against published stainless-route benchmarks (see the 'Calibration Basis' sheet); rows, headers, variables and formula shapes are unchanged from Grid 4.</t>
-        </is>
-      </c>
-    </row>
+          <t>Reference database of emission/energy formulas per process. Cells in Columns D-N are PLAIN TEXT formula ENTRIES (not live Excel formulas): x=virgin ratio, y=scrap ratio(=1-x); a-g = grid electricity source shares (Coal/Oil/Gas/Hydro/Wind/Solar/Nuclear, sum to 1); p=train share, q=road share(=1-p), used ONLY in the two Transport-related rows (Inbound&gt;Unloading/Inbound and Outbound&gt;Transport) — all other rows show N/A for p/q. See 'Grid Energy Mix Factors' sheet for a-g source factors. Only Scope 2 (Col P) varies with the energy mix; Scope 1, Scope 3(upstream), trace-gas columns and SEC do not. Column Q = Scope 3 UPSTREAM (GHG Protocol Cat. 1-8); downstream Cat. 9 is in Outbound &gt; Transport; Cat. 10-15 are in the 'Downstream Scope 3 (Product)' sheet. GWP basis: IPCC AR5 (100-yr). GRID 5: coefficients recalibrated against published stainless-route benchmarks (see the 'Calibration Basis' sheet); rows, headers, variables and formula shapes are unchanged from Grid 4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4" ht="45" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -739,7 +740,7 @@
     <row r="5" ht="190" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>RMHS</t>
+          <t>Inbound</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -874,7 +875,7 @@
     <row r="6" ht="140" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>RMHS</t>
+          <t>Inbound</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -999,7 +1000,7 @@
       </c>
       <c r="Z6" s="6" t="inlineStr">
         <is>
-          <t>Coefficients used in this row's formulas (Grid 5 calibration, RMHS materials-handling — replace with verified plant data before regulatory use):
+          <t>Coefficients used in this row's formulas (Grid 5 calibration, Inbound materials-handling — replace with verified plant data before regulatory use):
 EF_S1_virgin=0.001, EF_S1_scrap=0.001 tCO2e/t | EF_S2_virgin=0.0009, EF_S2_scrap=0.0009 tCO2e/t | EF_S3_virgin=0.0005, EF_S3_scrap=0.0005 tCO2e/t
 CO2_v=0.0006, CO2_s=0.0006 t/t | CH4_v=0.000001, CH4_s=0.000001 t/t (x28) | N2O_v=0.00000005, N2O_s=0.00000005 t/t (x265)
 HFC_v=0.00002, HFC_s=0.00002 tCO2e/t | PFC_v=0.000005, PFC_s=0.000005 tCO2e/t | SF6_v=0.00000002, SF6_s=0.00000002 t/t (x23500) | NF3_v=0.00000001, NF3_s=0.00000001 t/t (x16100)
@@ -1013,7 +1014,7 @@
     <row r="7" ht="140" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>RMHS</t>
+          <t>Inbound</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -1138,7 +1139,7 @@
       </c>
       <c r="Z7" s="6" t="inlineStr">
         <is>
-          <t>Coefficients used in this row's formulas (Grid 5 calibration, RMHS materials-handling — replace with verified plant data before regulatory use):
+          <t>Coefficients used in this row's formulas (Grid 5 calibration, Inbound materials-handling — replace with verified plant data before regulatory use):
 EF_S1_virgin=0.001, EF_S1_scrap=0.0015 tCO2e/t | EF_S2_virgin=0.0009, EF_S2_scrap=0.0012 tCO2e/t | EF_S3_virgin=0.0005, EF_S3_scrap=0.0006 tCO2e/t
 CO2_v=0.0006, CO2_s=0.0009 t/t | CH4_v=0.000001, CH4_s=0.0000015 t/t (x28) | N2O_v=0.00000005, N2O_s=0.00000007 t/t (x265)
 HFC_v=0.00002, HFC_s=0.00002 tCO2e/t | PFC_v=0.000005, PFC_s=0.000005 tCO2e/t | SF6_v=0.00000002, SF6_s=0.00000002 t/t (x23500) | NF3_v=0.00000001, NF3_s=0.00000001 t/t (x16100)
@@ -1152,7 +1153,7 @@
     <row r="8" ht="140" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>RMHS</t>
+          <t>Inbound</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -1277,12 +1278,12 @@
       </c>
       <c r="Z8" s="6" t="inlineStr">
         <is>
-          <t>Coefficients used in this row's formulas (Grid 5 calibration, RMHS materials-handling — replace with verified plant data before regulatory use):
+          <t>Coefficients used in this row's formulas (Grid 5 calibration, Inbound materials-handling — replace with verified plant data before regulatory use):
 EF_S1_virgin=0.0007, EF_S1_scrap=0.01225 tCO2e/t | EF_S2_virgin=0.0006, EF_S2_scrap=0.0168 tCO2e/t | EF_S3_virgin=0.0005, EF_S3_scrap=0.002 tCO2e/t
 CO2_v=0.000525, CO2_s=0.0098 t/t | CH4_v=0.00000035, CH4_s=0.000014 t/t (x28) | N2O_v=0.0000000175, N2O_s=0.0000007 t/t (x265)
 HFC_v=0.000012, HFC_s=0.000018 tCO2e/t | PFC_v=0.000003, PFC_s=0.000006 tCO2e/t | SF6_v=0.000000012, SF6_s=0.00000003 t/t (x23500) | NF3_v=0.000000006, NF3_s=0.000000006 t/t (x16100)
 SEC_virgin=0.0122647 GJ/t, SEC_scrap=0.244086 GJ/t.
-Basis: Hydraulic shears/balers, oxy-fuel/propane cutting torches for oversize scrap, magnetic separation. Virgin ferroalloys rarely need this stage, hence near-zero virgin-side factors; scrap side is by far the most energy/emission-intensive process in RMHS due to shearing and thermal cutting. Generalized across all sub-variations of this process (none specified yet) — illustrative literature-typical values, NOT plant-measured.
+Basis: Hydraulic shears/balers, oxy-fuel/propane cutting torches for oversize scrap, magnetic separation. Virgin ferroalloys rarely need this stage, hence near-zero virgin-side factors; scrap side is by far the most energy/emission-intensive process in Inbound due to shearing and thermal cutting. Generalized across all sub-variations of this process (none specified yet) — illustrative literature-typical values, NOT plant-measured.
 Scope 2 CUSTOMIZED: underlying electricity intensity backed out at the CEA-baseline reference (0.77 kg CO2e/kWh) = 0.779221 kWh/t (virgin), 21.8182 kWh/t (scrap). Actual Scope 2 now scales with your real grid mix (a-g) — see 'Grid Energy Mix Factors' sheet for per-source factors.
 Grid 5 calibration: Scrap shredding and baling draws ~20-25 kWh per tonne of scrap; yard diesel for mobile handling ~3-5 L/t. Grid 4 → Grid 5 (virgin/scrap): kWh/t 1.2987/36.3636 → 0.779221/21.8182; Scope 1 0.002/0.035 → 0.0007/0.01225; SEC GJ/t 0.02/0.65 → 0.0122647/0.244086.</t>
         </is>
@@ -1291,7 +1292,7 @@
     <row r="9" ht="140" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>RMHS</t>
+          <t>Inbound</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -1416,7 +1417,7 @@
       </c>
       <c r="Z9" s="6" t="inlineStr">
         <is>
-          <t>Coefficients used in this row's formulas (Grid 5 calibration, RMHS materials-handling — replace with verified plant data before regulatory use):
+          <t>Coefficients used in this row's formulas (Grid 5 calibration, Inbound materials-handling — replace with verified plant data before regulatory use):
 EF_S1_virgin=0.0032, EF_S1_scrap=0.008 tCO2e/t | EF_S2_virgin=0.0035, EF_S2_scrap=0.00525 tCO2e/t | EF_S3_virgin=0.0005, EF_S3_scrap=0.0008 tCO2e/t
 CO2_v=0.002, CO2_s=0.0064 t/t | CH4_v=0.000002, CH4_s=0.000008 t/t (x28) | N2O_v=0.00000008, N2O_s=0.0000004 t/t (x265)
 HFC_v=0.000007, HFC_s=0.000007 tCO2e/t | PFC_v=0.00000175, PFC_s=0.0000028 tCO2e/t | SF6_v=0.0000000105, SF6_s=0.0000000105 t/t (x23500) | NF3_v=0.0000000035, NF3_s=0.0000000035 t/t (x16100)
@@ -1430,7 +1431,7 @@
     <row r="10" ht="140" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>RMHS</t>
+          <t>Inbound</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
@@ -1555,7 +1556,7 @@
       </c>
       <c r="Z10" s="6" t="inlineStr">
         <is>
-          <t>Coefficients used in this row's formulas (Grid 5 calibration, RMHS materials-handling — replace with verified plant data before regulatory use):
+          <t>Coefficients used in this row's formulas (Grid 5 calibration, Inbound materials-handling — replace with verified plant data before regulatory use):
 EF_S1_virgin=0.004, EF_S1_scrap=0.0032 tCO2e/t | EF_S2_virgin=0.0036, EF_S2_scrap=0.0015 tCO2e/t | EF_S3_virgin=0.0003, EF_S3_scrap=0.0003 tCO2e/t
 CO2_v=0.0036, CO2_s=0.0028 t/t | CH4_v=0.000006, CH4_s=0.000004 t/t (x28) | N2O_v=0.00000028, N2O_s=0.0000002 t/t (x265)
 HFC_v=0.000006, HFC_s=0.000006 tCO2e/t | PFC_v=0.0000015, PFC_s=0.0000015 tCO2e/t | SF6_v=0.000000015, SF6_s=0.000000009 t/t (x23500) | NF3_v=0.000000003, NF3_s=0.000000003 t/t (x16100)
@@ -1569,7 +1570,7 @@
     <row r="11" ht="140" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>RMHS</t>
+          <t>Inbound</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
@@ -1694,7 +1695,7 @@
       </c>
       <c r="Z11" s="6" t="inlineStr">
         <is>
-          <t>Coefficients used in this row's formulas (Grid 5 calibration, RMHS materials-handling — replace with verified plant data before regulatory use):
+          <t>Coefficients used in this row's formulas (Grid 5 calibration, Inbound materials-handling — replace with verified plant data before regulatory use):
 EF_S1_virgin=0.001, EF_S1_scrap=0.002 tCO2e/t | EF_S2_virgin=0.0018, EF_S2_scrap=0.0036 tCO2e/t | EF_S3_virgin=0.0002, EF_S3_scrap=0.0002 tCO2e/t
 CO2_v=0.0008, CO2_s=0.0015 t/t | CH4_v=0.000001, CH4_s=0.000002 t/t (x28) | N2O_v=0.00000005, N2O_s=0.0000001 t/t (x265)
 HFC_v=0.000003, HFC_s=0.000003 tCO2e/t | PFC_v=0.0000009, PFC_s=0.0000009 tCO2e/t | SF6_v=0.000000015, SF6_s=0.000000024 t/t (x23500) | NF3_v=0.000000003, NF3_s=0.000000003 t/t (x16100)
@@ -1708,7 +1709,7 @@
     <row r="12" ht="140" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>RMHS</t>
+          <t>Inbound</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
@@ -1833,7 +1834,7 @@
       </c>
       <c r="Z12" s="6" t="inlineStr">
         <is>
-          <t>Coefficients used in this row's formulas (Grid 5 calibration, RMHS materials-handling — replace with verified plant data before regulatory use):
+          <t>Coefficients used in this row's formulas (Grid 5 calibration, Inbound materials-handling — replace with verified plant data before regulatory use):
 EF_S1_virgin=0.0005, EF_S1_scrap=0.0008 tCO2e/t | EF_S2_virgin=0.00375, EF_S2_scrap=0.0045 tCO2e/t | EF_S3_virgin=0.0001, EF_S3_scrap=0.0001 tCO2e/t
 CO2_v=0.0004, CO2_s=0.0006 t/t | CH4_v=0.0000005, CH4_s=0.0000008 t/t (x28) | N2O_v=0.00000002, N2O_s=0.00000003 t/t (x265)
 HFC_v=0.0000025, HFC_s=0.0000025 tCO2e/t | PFC_v=0.0000005, PFC_s=0.0000005 tCO2e/t | SF6_v=0.00000001, SF6_s=0.00000001 t/t (x23500) | NF3_v=0.0000000025, NF3_s=0.0000000025 t/t (x16100)
@@ -1977,7 +1978,7 @@
 CO2_v=0.003, CO2_s=0.006 t/t | CH4_v=0.000002, CH4_s=0.000005 t/t (x28) | N2O_v=0.0000001, N2O_s=0.0000002 t/t (x265)
 HFC_v=0.000007, HFC_s=0.000007 tCO2e/t | PFC_v=0.00000105, PFC_s=0.00000105 tCO2e/t | SF6_v=0.0000000175, SF6_s=0.0000000175 t/t (x23500) | NF3_v=0.0000000035, NF3_s=0.0000000035 t/t (x16100)
 SEC_virgin=0.105649 GJ/t, SEC_scrap=0.219481 GJ/t.
-Basis: Melt-shop-side charging operation (as distinct from RMHS's yard proportioning) — charge-crane/basket handling and scrap preheating (waste-heat/electric) prior to furnace charging. Illustrative literature-typical values — NOT plant-measured.
+Basis: Melt-shop-side charging operation (as distinct from Inbound's yard proportioning) — charge-crane/basket handling and scrap preheating (waste-heat/electric) prior to furnace charging. Illustrative literature-typical values — NOT plant-measured.
 Scope 2 CUSTOMIZED: underlying electricity intensity backed out at the CEA-baseline reference (0.77 kg CO2e/kWh) = 4.54545 kWh/t (virgin), 11.3636 kWh/t (scrap). Actual Scope 2 now scales with your real grid mix (a-g) — see 'Grid Energy Mix Factors' sheet for per-source factors.
 Grid 5 calibration: Scrap charging cranes and magnets: ~4-10 kWh/t. Grid 4 → Grid 5 (virgin/scrap): kWh/t 12.987/32.4675 → 4.54545/11.3636; SEC GJ/t 0.15/0.25 → 0.105649/0.219481.</t>
         </is>
@@ -10083,6 +10084,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -10219,6 +10221,7 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13" ht="55" customHeight="1">
       <c r="A13" s="10" t="inlineStr">
         <is>
@@ -10265,6 +10268,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -10427,6 +10431,7 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13" ht="70" customHeight="1">
       <c r="A13" s="14" t="inlineStr">
         <is>
@@ -10434,6 +10439,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15" ht="65" customHeight="1">
       <c r="A15" s="10" t="inlineStr">
         <is>
@@ -10492,6 +10498,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="17" t="inlineStr">
         <is>
@@ -10815,6 +10822,7 @@
         </is>
       </c>
     </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" s="18" t="inlineStr">
         <is>
@@ -10898,7 +10906,7 @@
       </c>
       <c r="B25" s="16" t="inlineStr">
         <is>
-          <t>RMHS</t>
+          <t>Inbound</t>
         </is>
       </c>
       <c r="C25" s="16" t="inlineStr">
@@ -10933,7 +10941,7 @@
       </c>
       <c r="B26" s="16" t="inlineStr">
         <is>
-          <t>RMHS</t>
+          <t>Inbound</t>
         </is>
       </c>
       <c r="C26" s="16" t="inlineStr">
@@ -11000,7 +11008,7 @@
       </c>
       <c r="B27" s="16" t="inlineStr">
         <is>
-          <t>RMHS</t>
+          <t>Inbound</t>
         </is>
       </c>
       <c r="C27" s="16" t="inlineStr">
@@ -11067,7 +11075,7 @@
       </c>
       <c r="B28" s="16" t="inlineStr">
         <is>
-          <t>RMHS</t>
+          <t>Inbound</t>
         </is>
       </c>
       <c r="C28" s="16" t="inlineStr">
@@ -11134,7 +11142,7 @@
       </c>
       <c r="B29" s="16" t="inlineStr">
         <is>
-          <t>RMHS</t>
+          <t>Inbound</t>
         </is>
       </c>
       <c r="C29" s="16" t="inlineStr">
@@ -11201,7 +11209,7 @@
       </c>
       <c r="B30" s="16" t="inlineStr">
         <is>
-          <t>RMHS</t>
+          <t>Inbound</t>
         </is>
       </c>
       <c r="C30" s="16" t="inlineStr">
@@ -11268,7 +11276,7 @@
       </c>
       <c r="B31" s="16" t="inlineStr">
         <is>
-          <t>RMHS</t>
+          <t>Inbound</t>
         </is>
       </c>
       <c r="C31" s="16" t="inlineStr">
@@ -11335,7 +11343,7 @@
       </c>
       <c r="B32" s="16" t="inlineStr">
         <is>
-          <t>RMHS</t>
+          <t>Inbound</t>
         </is>
       </c>
       <c r="C32" s="16" t="inlineStr">

</xml_diff>